<commit_message>
Docs: documenta Desayuno y tiempos de comida; actualiza requerimientos (RF-68 a RF-72) y mapa del sistema
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Requerimientos_Oasis.xlsx
+++ b/docs/Requerimientos_Oasis.xlsx
@@ -524,13 +524,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B14"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -545,6 +546,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -566,6 +568,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -604,7 +607,8 @@
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>• Ver también docs/MAPA_DEL_SISTEMA.md en este mismo repositorio para el detalle técnico completo (rutas, modelo de datos, reglas de negocio).</t>
+          <t>• Actualización 2026-09-20: se agregó la categoría Desayuno y la selección de 1, 2 o 3 tiempos de comida por pedido (RF-68 a RF-72, notas '[Actualizado 2026-09-20]' en RF-10, 16, 19, 20, 23, 25, 34, 35 y 51). Ver docs/TIEMPOS_DE_COMIDA_DESAYUNO.md.
+• Ver también docs/MAPA_DEL_SISTEMA.md en este mismo repositorio para el detalle técnico completo (rutas, modelo de datos, reglas de negocio).</t>
         </is>
       </c>
     </row>
@@ -619,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1029,7 +1033,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>El sistema debe permitir asignar un perfil de macros (proteína/carbohidrato) separado para almuerzo y para cena.</t>
+          <t>El sistema debe permitir asignar un perfil de macros (proteína/carbohidrato) separado para desayuno (opcional), almuerzo y cena.</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1044,7 +1048,8 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Los valores son unidades enteras, no gramos ni calorías.</t>
+          <t>Los valores son unidades enteras, no gramos ni calorías.
+[Actualizado 2026-09-20] Se agregó el perfil de desayuno (clients.breakfast_macro_profile_id, opcional para no bloquear clientes existentes). Ver RF-68.</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1244,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>El sistema debe permitir crear un pedido semanal para un cliente, asociado a una plantilla o a selección manual de recetas por día.</t>
+          <t>El sistema debe permitir crear un pedido semanal para un cliente, asociado a una plantilla o a selección manual de recetas por día, eligiendo uno, dos o los tres tiempos de comida (desayuno, almuerzo, cena).</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1254,7 +1259,8 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Asistente de 5 pasos: Cliente → Menú → Ajustes → Pago → Confirmar.</t>
+          <t>Asistente de 5 pasos: Cliente → Menú → Ajustes → Pago → Confirmar.
+[Actualizado 2026-09-20] El paso Menú ahora es de selección múltiple de tiempos de comida (ver RF-69) y el paso Ajustes muestra macros por cada tiempo (RF-70).</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1369,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-09-20] Con más de un tiempo de comida en el pedido (antes solo 'both') se sugiere ruta 'complete'; un solo tiempo → 'individual'.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1383,7 +1393,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>El sistema debe permitir sobrescribir los valores de macro de un día/comida específicos sin alterar el perfil base del cliente.</t>
+          <t>El sistema debe permitir sobrescribir los valores de macro de un día/comida específicos (por tiempo de comida) sin alterar el perfil base del cliente.</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -1396,7 +1406,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-09-20] Cada tiempo del pedido tiene su propio panel de override por día.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1490,7 +1504,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>El sistema debe permitir modificar un pedido ya creado (menú, cantidades, macros).</t>
+          <t>El sistema debe permitir modificar un pedido ya creado (menú, cantidades, macros de cada tiempo de comida).</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1505,7 +1519,8 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>La edición borra y vuelve a insertar días/detalles en vez de calcular diferencias.</t>
+          <t>La edición borra y vuelve a insertar días/detalles en vez de calcular diferencias.
+[Actualizado 2026-09-20] La edición carga y guarda los macros de TODOS los tiempos del pedido; cada receta se guarda con los macros de su tiempo (RF-70). En main el tiempo de cada receta se infiere por los macros aplicados; en Fase_2 se lee de order_day_details.meal_type.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1588,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-09-20] Express admite Desayuno, Almuerzo o Cena (macros del perfil del cliente o estándar).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -1877,7 +1896,7 @@
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>El sistema debe permitir crear plantillas reutilizables que asignen recetas a cada día de la semana para almuerzo o cena.</t>
+          <t>El sistema debe permitir crear plantillas reutilizables que asignen recetas a cada día de la semana para desayuno, almuerzo o cena.</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -1890,7 +1909,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-09-20] Nuevo tipo de plantilla 'Desayuno' (meal_type='Breakfast'), con semana del mes y anulación semanal para el portal (RF-71).</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -1923,7 +1946,11 @@
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G39" s="8" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>[Actualizado 2026-09-20] Al elegir varios tiempos, se preselecciona la plantilla de la semana en curso de cada uno y se combinan sus recetas; cada receta queda ligada a su tiempo de comida.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -2481,7 +2508,8 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Página Main.</t>
+          <t>Página Main.
+[Actualizado 2026-09-20] La dona de clasificación incluye Desayuno y 'Combinado' (pedidos con más de un tiempo, incluidos los 'both' que antes no se contaban).</t>
         </is>
       </c>
     </row>
@@ -3070,6 +3098,191 @@
       <c r="G71" s="8" t="inlineStr">
         <is>
           <t>[Nuevo 2026-08-17, a petición del usuario] Payments.jsx: filtro de Tipo de pago, al valor 'monthly', además de igualar payment_type aplica status in (pending, paid) AND closed_at IS NULL AND órdenes vinculadas &lt; 4, con un badge visible ('Mostrando solo mensuales vigentes con órdenes disponibles'). Pensado para auditar de un vistazo cuál es el pago mensual activo de cada cliente y detectar fragmentación (más de un pago vigente simultáneo para el mismo cliente) sin consultar la base de datos directamente — ver project-monthly-payment-fragmentation en memoria. Verificado con Playwright contra producción: con este filtro + pestaña Historial se confirmaron 11 pagos mensuales vigentes, uno por cliente, sin duplicados; el filtro destapó un pago suelto real (Erick Vásquez #19, 2/4, de junio) que se había quedado sin cerrar en una limpieza de datos anterior — se cerró en el momento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>RF-68</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>Clientes</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Perfil de macros de desayuno (opcional)</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>El sistema debe permitir definir opcionalmente un perfil de macros de desayuno por cliente personal (alta y edición). Si se completa un campo, ambos son obligatorios; si está vacío, el cliente no tiene perfil de desayuno y los pedidos parten de macros estándar.</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-09-20, a petición del usuario] AddCustomer.jsx, CustomerTable, CustomerDetailModal, customer.jsx. Columna clients.breakfast_macro_profile_id (migración 20260920_breakfast_category.sql, aplicada en producción). plan_type = 'estandar' solo si todos los tiempos del cliente son estándar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>RF-69</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Elegir 1, 2 o los 3 tiempos de comida por pedido</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>El sistema debe permitir que un pedido personal incluya uno, dos o los tres tiempos de comida (desayuno, almuerzo, cena), elegidos con interruptores en el paso Menú; 'Almuerzo + Cena' equivale al antiguo 'Ambos'.</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-09-20, a petición del usuario] orders.classification: tiempo suelto, 'both' (Almuerzo + Cena, legado) o combinación con '+' en orden canónico (Breakfast+Lunch+Dinner). Helpers en orderUtils.js (mealTypesOf, classificationOf). Badges/etiquetas en Producción, Empaque, Entrega, Pagos y Dashboard. Ver docs/TIEMPOS_DE_COMIDA_DESAYUNO.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>RF-70</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Macros obligatorios y aplicados por tiempo de comida</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Por cada tiempo de comida elegido, el asistente y la edición deben mostrar (obligatoriamente) su panel de macros; cada receta debe guardarse con los macros de su propio tiempo. Sin perfil del cliente, el tiempo arranca en macros estándar.</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-09-20, a petición del usuario] El snapshot de macros del pedido corresponde al primer tiempo. Corrige que en pedidos 'both' todas las recetas salían con macros de almuerzo. En Fase_2 el tiempo por receta se persiste en order_day_details.meal_type (migración 20260921).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>RF-71</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>Menús y Plantillas</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Plantillas y plantilla semanal para desayuno</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>El sistema debe permitir crear plantillas de desayuno y anular por tiempo de comida la plantilla semanal que aplica el portal de clientes.</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-09-20, a petición del usuario] AddTemplate, TemplateCard, WeeklyTemplateOverride; portal_template_overrides.meal_type admite 'Breakfast'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>RF-72</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>Portal de Clientes</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Elegir uno o varios tiempos de comida en el portal</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>El portal debe mostrar los macros de cada tiempo del cliente y permitirle armar su pedido semanal con uno o varios tiempos; si solo tiene macros de un tiempo, se selecciona automáticamente.</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="G76" s="8" t="inlineStr">
+        <is>
+          <t>[Nuevo 2026-09-20, a petición del usuario] CustomerPortal.jsx, PortalOrderSummary.jsx y RPC portal_get_client / portal_get_menu_options / portal_submit_order actualizadas. Probado por RPC y UI en staging; no probado en el navegador contra producción.</t>
         </is>
       </c>
     </row>
@@ -3948,7 +4161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4620,6 +4833,168 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Corregido (incidental)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>src/components/AddOrder.jsx — macro_profile_snapshot_id</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>La consulta de clientes solo traía el perfil embebido (no la columna *_macro_profile_id), por lo que el snapshot del pedido se guardaba siempre en null para almuerzo y cena.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Ahora se toma de selectedClient[...].id_macro_profile. Verificado con Playwright en staging (2026-09-20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Corregido (incidental)</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>src/hooks/useDashboardData.js</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>El conteo por clasificación ignoraba los pedidos "both" (62 en producción).</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Ahora cuentan como "Combinado" junto con el resto de combinaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Corregido (incidental)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>src/components/orders/OrderBlock.jsx</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Rotulaba "both" como "Familiar" en Detalle de cliente → Órdenes (hallazgo colateral del 2026-08-18).</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Ahora usa mealLabel/classificationBadge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente (a considerar)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Riesgo de despliegue</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>supabase/migrations 20260818_* / 20260920 / 20260921</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>portal_submit_order tiene versiones distintas por rama: producción usa la de 20260920 (sin meal_type por detalle); Fase_2 usa 20260921.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Al llevar Fase_2 a producción aplicar 20260818 y luego 20260921; si solo se aplica la 0818, el portal pierde el soporte de desayuno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente (a considerar)</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Limitación</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>src/components/EditOrder.jsx (rama main)</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Sin order_day_details.meal_type en producción, el tiempo de comida de cada receta existente se infiere comparando los macros aplicados; es ambiguo si dos tiempos tienen macros idénticos.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Se resuelve al desplegar Fase_2 (lee meal_type). Sin impacto en pedidos de un solo tiempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente (observado, no tocado)</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Deuda técnica</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>src/components/EditOrder.jsx</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>La edición borra y reinserta días/detalles y no recarga los overrides de ingredientes existentes (order_day_recipe_overrides), por lo que se pierden al guardar.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Preexistente; no relacionado con desayunos. Conviene evaluarlo por separado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>